<commit_message>
[20 26] update excel_zad2 add chart
</commit_message>
<xml_diff>
--- a/day_20_31_08_2025/xlsxwriter6.xlsx
+++ b/day_20_31_08_2025/xlsxwriter6.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>Witaj1</t>
   </si>
@@ -23,6 +23,12 @@
   </si>
   <si>
     <t>Witaj 3</t>
+  </si>
+  <si>
+    <t>Styczeń</t>
+  </si>
+  <si>
+    <t>Luty</t>
   </si>
 </sst>
 </file>
@@ -107,6 +113,154 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Sprzedaż</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Arkusz1!A11</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:cat>
+            <c:strRef>
+              <c:f>Arkusz1!B10:C10</c:f>
+              <c:strCache>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>Styczeń</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Luty</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Arkusz1!B11:C11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>150</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="50010001"/>
+        <c:axId val="50010002"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="50010001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Os X</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+        </c:title>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50010002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="50010002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Os Y</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50010001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
@@ -145,6 +299,36 @@
         </a:prstGeom>
       </xdr:spPr>
     </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -435,38 +619,54 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1">
+    <row r="3" spans="1:3">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1">
+    <row r="4" spans="1:3">
       <c r="A4" s="2">
         <v>42656</v>
       </c>
     </row>
-    <row r="5" spans="1:1">
+    <row r="5" spans="1:3">
       <c r="A5" s="3">
         <v>3.3333333</v>
       </c>
     </row>
-    <row r="6" spans="1:1">
+    <row r="6" spans="1:3">
       <c r="A6">
         <f>SUM(A4, 2)</f>
         <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="B10" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="B11">
+        <v>100</v>
+      </c>
+      <c r="C11">
+        <v>150</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[20 27] update excel_zad2 add chart fix
</commit_message>
<xml_diff>
--- a/day_20_31_08_2025/xlsxwriter6.xlsx
+++ b/day_20_31_08_2025/xlsxwriter6.xlsx
@@ -145,7 +145,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Arkusz1!A11</c:f>
+              <c:f>Arkusz1!A30</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
               </c:strCache>
@@ -153,7 +153,7 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>Arkusz1!B10:C10</c:f>
+              <c:f>Arkusz1!B20:C20</c:f>
               <c:strCache>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
@@ -167,7 +167,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Arkusz1!B11:C11</c:f>
+              <c:f>Arkusz1!B21:C21</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
@@ -265,16 +265,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>28</xdr:col>
-      <xdr:colOff>495300</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>247650</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -291,8 +291,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1219200" y="0"/>
-          <a:ext cx="16344900" cy="7677150"/>
+          <a:off x="3048000" y="0"/>
+          <a:ext cx="8172450" cy="3838575"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -619,53 +619,53 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:1">
       <c r="A2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:1">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:1">
       <c r="A4" s="2">
         <v>42656</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:1">
       <c r="A5" s="3">
         <v>3.3333333</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:1">
       <c r="A6">
         <f>SUM(A4, 2)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
-      <c r="B10" t="s">
+    <row r="20" spans="2:3">
+      <c r="B20" t="s">
         <v>3</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C20" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
-      <c r="B11">
+    <row r="21" spans="2:3">
+      <c r="B21">
         <v>100</v>
       </c>
-      <c r="C11">
+      <c r="C21">
         <v>150</v>
       </c>
     </row>

</xml_diff>